<commit_message>
File mẫu Biên bản nhập hàng: "Fit to 1 page wide" thay vì tỉ lệ in cố định 89%
Mẫu trước đây set cứng tỉ lệ in scale=89% — không đủ để cột M (Ghi chú) nằm
gọn trong khổ giấy A4 ngang khi in thật, khiến cột L/M (Tình trạng/Ghi chú)
bị tách hẳn sang 1 khối trang riêng biệt (ảnh người dùng gửi: đánh số "Page
5", tách khỏi mạch trang 1-4 của các cột A-K).

Đổi sang "Fit to 1 page wide" (sheetPr.pageSetUpPr fitToPage="1" +
pageSetup fitToWidth="1" fitToHeight="0", bỏ scale="89" cố định) — Excel tự
co tỉ lệ in vừa đúng 1 trang ngang cho tất cả các cột A-M, không phụ thuộc
1 con số % cố định (vốn không tính đến độ rộng cột M thật sự cần).

Thêm test xác nhận cấu hình mới giữ nguyên qua fillReceiptTemplate().

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013X5GNx7RrqCSGurkhHGXN6
</commit_message>
<xml_diff>
--- a/public/templates/BIEN_BAN_NHAP_HANG.xlsx
+++ b/public/templates/BIEN_BAN_NHAP_HANG.xlsx
@@ -864,6 +864,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F379C3-B36E-FA46-90ED-3D8D3F44DE72}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="31.5" customHeight="1"/>
   <cols>
@@ -1393,7 +1396,7 @@
     <mergeCell ref="F13:G13"/>
   </mergeCells>
   <pageMargins left="0.16" right="0.12" top="0.12" bottom="0.12" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="89" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="28" max="16383" man="1"/>

</xml_diff>